<commit_message>
improve initial voltage reaching
</commit_message>
<xml_diff>
--- a/files/316_Resistivity_curve_literature.xlsx
+++ b/files/316_Resistivity_curve_literature.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TDS\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TDS\PycharmProjects\TDS_data_acquisition\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="820" windowWidth="46980" windowHeight="24000"/>
+    <workbookView xWindow="1560" yWindow="825" windowWidth="46980" windowHeight="24000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -187,7 +187,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="de-DE"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -276,40 +276,40 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>20.937716957867121</c:v>
+                  <c:v>10.599719209920231</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>23.201253926285187</c:v>
+                  <c:v>11.745634800181875</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>25.46479089470326</c:v>
+                  <c:v>12.891550390443525</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27.445385742069064</c:v>
+                  <c:v>13.894226531922463</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28.860096347330359</c:v>
+                  <c:v>14.610423775835994</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>29.14303846838261</c:v>
+                  <c:v>14.753663224618697</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>29.425980589434872</c:v>
+                  <c:v>14.896902673401401</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>30.557749073643908</c:v>
+                  <c:v>15.469860468532227</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>31.689517557852934</c:v>
+                  <c:v>16.042818263663047</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>32.538343921009712</c:v>
+                  <c:v>16.472536610011169</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>33.104228163114236</c:v>
+                  <c:v>16.759015507576581</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>33.953054526271011</c:v>
+                  <c:v>17.188733853924699</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -387,7 +387,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="de-DE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1210225487"/>
@@ -449,7 +449,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="de-DE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="366255760"/>
@@ -497,7 +497,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="de-DE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1423,14 +1423,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:I14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="5" max="5" width="21.15234375" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" customWidth="1"/>
     <col min="6" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
-    <col min="9" max="9" width="13.61328125" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9">
@@ -1472,21 +1472,21 @@
       </c>
       <c r="D3">
         <f>C3/1000000 * 10 *$I$3 /$H$7</f>
-        <v>20.937716957867121</v>
+        <v>10.599719209920231</v>
       </c>
       <c r="E3">
         <f>(D4-D3)/(A4-A3) *1000</f>
-        <v>11.31768484209033</v>
+        <v>5.7295779513082223</v>
       </c>
       <c r="F3">
         <f>E3/1000 / D3</f>
-        <v>5.4054054054054022E-4</v>
+        <v>5.4054054054053957E-4</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I3">
-        <v>80</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1502,15 +1502,15 @@
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D14" si="1">C4/1000000 * 10 *$I$3 /$H$7</f>
-        <v>23.201253926285187</v>
+        <v>11.745634800181875</v>
       </c>
       <c r="E4">
         <f t="shared" ref="E4:E13" si="2">(D5-D4)/(A5-A4) *1000</f>
-        <v>11.317684842090365</v>
+        <v>5.729577951308249</v>
       </c>
       <c r="F4">
         <f t="shared" ref="F4:F13" si="3">E4/1000 / D4</f>
-        <v>4.8780487804878184E-4</v>
+        <v>4.8780487804878195E-4</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1526,15 +1526,15 @@
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>25.46479089470326</v>
+        <v>12.891550390443525</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>9.9029742368290208</v>
+        <v>5.0133807073946901</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>3.8888888888888789E-4</v>
+        <v>3.8888888888888778E-4</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1550,11 +1550,11 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>27.445385742069064</v>
+        <v>13.894226531922463</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>9.4314040350752979</v>
+        <v>4.7746482927568694</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
@@ -1577,19 +1577,19 @@
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>28.860096347330359</v>
+        <v>14.610423775835994</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>5.6588424210450228</v>
+        <v>2.8647889756540579</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.9607843137254397E-4</v>
+        <v>1.9607843137254503E-4</v>
       </c>
       <c r="H7">
         <f>(H3/1000)^2 * PI() /4</f>
-        <v>2.8274333882308137E-3</v>
+        <v>1.2566370614359172E-3</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1605,15 +1605,15 @@
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>29.14303846838261</v>
+        <v>14.753663224618697</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>5.6588424210452359</v>
+        <v>2.8647889756540934</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.9417475728155577E-4</v>
+        <v>1.9417475728155189E-4</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1629,15 +1629,15 @@
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>29.425980589434872</v>
+        <v>14.896902673401401</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>7.5451232280602429</v>
+        <v>3.8197186342055049</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>2.5641025641025706E-4</v>
+        <v>2.564102564102576E-4</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1653,15 +1653,15 @@
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>30.557749073643908</v>
+        <v>15.469860468532227</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>5.6588424210451294</v>
+        <v>2.8647889756541023</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.851851851851839E-4</v>
+        <v>1.8518518518518428E-4</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1677,15 +1677,15 @@
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>31.689517557852934</v>
+        <v>16.042818263663047</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>4.2441318157838914</v>
+        <v>2.1485917317406056</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.3392857142857195E-4</v>
+        <v>1.339285714285726E-4</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1701,15 +1701,15 @@
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>32.538343921009712</v>
+        <v>16.472536610011169</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>2.829421210522618</v>
+        <v>1.4323944878270645</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>8.6956521739131484E-5</v>
+        <v>8.6956521739130807E-5</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1725,15 +1725,15 @@
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>33.104228163114236</v>
+        <v>16.759015507576581</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>4.2441318157838737</v>
+        <v>2.1485917317405878</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>1.2820512820512812E-4</v>
+        <v>1.2820512820512823E-4</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>33.953054526271011</v>
+        <v>17.188733853924699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>